<commit_message>
Including State Space Solver
</commit_message>
<xml_diff>
--- a/config/default.xlsx
+++ b/config/default.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/f215465b21b5e6e2/Studium/34_Github/TherMOS/config/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="18" documentId="13_ncr:1_{1A1B7590-5493-4A3C-A7B2-6BC5FABEA6F3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{804777F3-FA3C-4C1C-964C-7E219E944C85}"/>
+  <xr:revisionPtr revIDLastSave="22" documentId="13_ncr:1_{1A1B7590-5493-4A3C-A7B2-6BC5FABEA6F3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{DD45966B-4162-4967-BA4D-0AEEDCB1E41B}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="30936" windowHeight="16896" activeTab="1" xr2:uid="{DB7D2548-4471-4992-93B1-3EC0BA66F7EA}"/>
   </bookViews>
@@ -40,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="393" uniqueCount="190">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="389" uniqueCount="189">
   <si>
     <t>#</t>
   </si>
@@ -279,12 +279,6 @@
   </si>
   <si>
     <t>Solver Init</t>
-  </si>
-  <si>
-    <t>N4SID Init</t>
-  </si>
-  <si>
-    <t>N4SID Stability</t>
   </si>
   <si>
     <t>ss</t>
@@ -653,6 +647,9 @@
   </si>
   <si>
     <t>dy</t>
+  </si>
+  <si>
+    <t>Stability</t>
   </si>
 </sst>
 </file>
@@ -1204,6 +1201,10 @@
     </ext>
   </extLst>
 </styleSheet>
+</file>
+
+<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
+<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -1697,19 +1698,19 @@
     </row>
     <row r="2" spans="1:7" ht="58.2" thickTop="1" x14ac:dyDescent="0.3">
       <c r="A2" s="13" t="s">
-        <v>99</v>
+        <v>97</v>
       </c>
       <c r="B2" s="26" t="s">
         <v>63</v>
       </c>
       <c r="C2" s="46" t="s">
-        <v>120</v>
+        <v>118</v>
       </c>
       <c r="D2" s="26" t="s">
-        <v>80</v>
+        <v>78</v>
       </c>
       <c r="E2" s="26" t="s">
-        <v>119</v>
+        <v>117</v>
       </c>
       <c r="F2" s="6">
         <v>1</v>
@@ -1720,13 +1721,13 @@
     </row>
     <row r="3" spans="1:7" ht="57.6" x14ac:dyDescent="0.3">
       <c r="A3" s="13" t="s">
-        <v>100</v>
+        <v>98</v>
       </c>
       <c r="B3" s="26" t="s">
         <v>63</v>
       </c>
       <c r="C3" s="5" t="s">
-        <v>116</v>
+        <v>114</v>
       </c>
       <c r="D3" s="26" t="s">
         <v>22</v>
@@ -1743,16 +1744,16 @@
     </row>
     <row r="4" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A4" s="13" t="s">
-        <v>101</v>
+        <v>99</v>
       </c>
       <c r="B4" s="26" t="s">
         <v>63</v>
       </c>
       <c r="C4" s="5" t="s">
-        <v>117</v>
+        <v>115</v>
       </c>
       <c r="D4" s="26" t="s">
-        <v>136</v>
+        <v>134</v>
       </c>
       <c r="E4" s="26" t="s">
         <v>49</v>
@@ -1766,16 +1767,16 @@
     </row>
     <row r="5" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A5" s="13" t="s">
-        <v>185</v>
+        <v>183</v>
       </c>
       <c r="B5" s="26" t="s">
         <v>63</v>
       </c>
       <c r="C5" s="5" t="s">
-        <v>187</v>
+        <v>185</v>
       </c>
       <c r="D5" s="26" t="s">
-        <v>188</v>
+        <v>186</v>
       </c>
       <c r="E5" s="26" t="s">
         <v>49</v>
@@ -1784,21 +1785,21 @@
         <v>0.01</v>
       </c>
       <c r="G5" s="29" t="s">
-        <v>115</v>
+        <v>113</v>
       </c>
     </row>
     <row r="6" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A6" s="13" t="s">
-        <v>186</v>
+        <v>184</v>
       </c>
       <c r="B6" s="26" t="s">
         <v>63</v>
       </c>
       <c r="C6" s="5" t="s">
+        <v>185</v>
+      </c>
+      <c r="D6" s="26" t="s">
         <v>187</v>
-      </c>
-      <c r="D6" s="26" t="s">
-        <v>189</v>
       </c>
       <c r="E6" s="26" t="s">
         <v>49</v>
@@ -1807,24 +1808,24 @@
         <v>0.01</v>
       </c>
       <c r="G6" s="29" t="s">
-        <v>115</v>
+        <v>113</v>
       </c>
     </row>
     <row r="7" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A7" s="13" t="s">
-        <v>102</v>
+        <v>100</v>
       </c>
       <c r="B7" s="26" t="s">
         <v>63</v>
       </c>
       <c r="C7" s="5" t="s">
-        <v>118</v>
+        <v>116</v>
       </c>
       <c r="D7" s="26" t="s">
-        <v>137</v>
+        <v>135</v>
       </c>
       <c r="E7" s="26" t="s">
-        <v>119</v>
+        <v>117</v>
       </c>
       <c r="F7" s="6">
         <v>0</v>
@@ -2099,16 +2100,16 @@
     </row>
     <row r="2" spans="1:7" ht="43.8" thickTop="1" x14ac:dyDescent="0.3">
       <c r="A2" s="13" t="s">
-        <v>103</v>
+        <v>101</v>
       </c>
       <c r="B2" s="26" t="s">
         <v>63</v>
       </c>
       <c r="C2" s="5" t="s">
-        <v>105</v>
+        <v>103</v>
       </c>
       <c r="D2" s="26" t="s">
-        <v>109</v>
+        <v>107</v>
       </c>
       <c r="E2" s="26" t="s">
         <v>48</v>
@@ -2122,16 +2123,16 @@
     </row>
     <row r="3" spans="1:7" ht="72" x14ac:dyDescent="0.3">
       <c r="A3" s="13" t="s">
-        <v>104</v>
+        <v>102</v>
       </c>
       <c r="B3" s="26" t="s">
         <v>63</v>
       </c>
       <c r="C3" s="5" t="s">
-        <v>106</v>
+        <v>104</v>
       </c>
       <c r="D3" s="26" t="s">
-        <v>110</v>
+        <v>108</v>
       </c>
       <c r="E3" s="26" t="s">
         <v>48</v>
@@ -2145,177 +2146,177 @@
     </row>
     <row r="4" spans="1:7" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A4" s="13" t="s">
-        <v>107</v>
+        <v>105</v>
       </c>
       <c r="B4" s="26" t="s">
         <v>63</v>
       </c>
       <c r="C4" s="5" t="s">
-        <v>108</v>
+        <v>106</v>
       </c>
       <c r="D4" s="26" t="s">
-        <v>111</v>
+        <v>109</v>
       </c>
       <c r="E4" s="26" t="s">
-        <v>112</v>
+        <v>110</v>
       </c>
       <c r="F4" s="11">
         <v>0</v>
       </c>
       <c r="G4" s="29" t="s">
-        <v>115</v>
+        <v>113</v>
       </c>
     </row>
     <row r="5" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A5" s="13" t="s">
-        <v>121</v>
+        <v>119</v>
       </c>
       <c r="B5" s="26" t="s">
         <v>63</v>
       </c>
       <c r="C5" s="5" t="s">
-        <v>133</v>
+        <v>131</v>
       </c>
       <c r="D5" s="26" t="s">
-        <v>127</v>
+        <v>125</v>
       </c>
       <c r="E5" s="26" t="s">
-        <v>112</v>
+        <v>110</v>
       </c>
       <c r="F5" s="11">
         <v>0</v>
       </c>
       <c r="G5" s="29" t="s">
-        <v>115</v>
+        <v>113</v>
       </c>
     </row>
     <row r="6" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A6" s="13" t="s">
-        <v>122</v>
+        <v>120</v>
       </c>
       <c r="B6" s="26" t="s">
         <v>63</v>
       </c>
       <c r="C6" s="5" t="s">
-        <v>135</v>
+        <v>133</v>
       </c>
       <c r="D6" s="26" t="s">
-        <v>128</v>
+        <v>126</v>
       </c>
       <c r="E6" s="26" t="s">
-        <v>112</v>
+        <v>110</v>
       </c>
       <c r="F6" s="11">
         <v>0</v>
       </c>
       <c r="G6" s="29" t="s">
-        <v>115</v>
+        <v>113</v>
       </c>
     </row>
     <row r="7" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A7" s="13" t="s">
-        <v>123</v>
+        <v>121</v>
       </c>
       <c r="B7" s="26" t="s">
         <v>63</v>
       </c>
       <c r="C7" s="5" t="s">
-        <v>134</v>
+        <v>132</v>
       </c>
       <c r="D7" s="26" t="s">
-        <v>129</v>
+        <v>127</v>
       </c>
       <c r="E7" s="26" t="s">
-        <v>112</v>
+        <v>110</v>
       </c>
       <c r="F7" s="11">
         <v>0</v>
       </c>
       <c r="G7" s="29" t="s">
-        <v>115</v>
+        <v>113</v>
       </c>
     </row>
     <row r="8" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A8" s="13" t="s">
-        <v>124</v>
+        <v>122</v>
       </c>
       <c r="B8" s="26" t="s">
         <v>63</v>
       </c>
       <c r="C8" s="5" t="s">
-        <v>133</v>
+        <v>131</v>
       </c>
       <c r="D8" s="26" t="s">
-        <v>130</v>
+        <v>128</v>
       </c>
       <c r="E8" s="26" t="s">
-        <v>112</v>
+        <v>110</v>
       </c>
       <c r="F8" s="11">
         <v>0</v>
       </c>
       <c r="G8" s="29" t="s">
-        <v>115</v>
+        <v>113</v>
       </c>
     </row>
     <row r="9" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A9" s="13" t="s">
-        <v>125</v>
+        <v>123</v>
       </c>
       <c r="B9" s="26" t="s">
         <v>63</v>
       </c>
       <c r="C9" s="5" t="s">
-        <v>135</v>
+        <v>133</v>
       </c>
       <c r="D9" s="26" t="s">
-        <v>131</v>
+        <v>129</v>
       </c>
       <c r="E9" s="26" t="s">
-        <v>112</v>
+        <v>110</v>
       </c>
       <c r="F9" s="11">
         <v>0</v>
       </c>
       <c r="G9" s="29" t="s">
-        <v>115</v>
+        <v>113</v>
       </c>
     </row>
     <row r="10" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A10" s="13" t="s">
-        <v>126</v>
+        <v>124</v>
       </c>
       <c r="B10" s="26" t="s">
         <v>63</v>
       </c>
       <c r="C10" s="5" t="s">
-        <v>134</v>
+        <v>132</v>
       </c>
       <c r="D10" s="26" t="s">
-        <v>132</v>
+        <v>130</v>
       </c>
       <c r="E10" s="26" t="s">
-        <v>112</v>
+        <v>110</v>
       </c>
       <c r="F10" s="11">
         <v>0</v>
       </c>
       <c r="G10" s="29" t="s">
-        <v>115</v>
+        <v>113</v>
       </c>
     </row>
     <row r="11" spans="1:7" ht="86.4" x14ac:dyDescent="0.3">
       <c r="A11" s="13" t="s">
-        <v>113</v>
+        <v>111</v>
       </c>
       <c r="B11" s="26" t="s">
         <v>63</v>
       </c>
       <c r="C11" s="5" t="s">
-        <v>177</v>
+        <v>175</v>
       </c>
       <c r="D11" s="26" t="s">
-        <v>114</v>
+        <v>112</v>
       </c>
       <c r="E11" s="26" t="s">
         <v>48</v>
@@ -2495,7 +2496,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{799FBFCB-8244-4B83-8CC9-EBD2890613E5}">
-  <dimension ref="A1:G43"/>
+  <dimension ref="A1:G42"/>
   <sheetFormatPr defaultColWidth="9.109375" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="29.33203125" bestFit="1" customWidth="1"/>
@@ -2536,7 +2537,7 @@
         <v>63</v>
       </c>
       <c r="C2" s="8" t="s">
-        <v>162</v>
+        <v>160</v>
       </c>
       <c r="D2" s="28" t="s">
         <v>65</v>
@@ -2559,7 +2560,7 @@
         <v>63</v>
       </c>
       <c r="C3" s="5" t="s">
-        <v>160</v>
+        <v>158</v>
       </c>
       <c r="D3" s="26" t="s">
         <v>20</v>
@@ -2582,7 +2583,7 @@
         <v>63</v>
       </c>
       <c r="C4" s="5" t="s">
-        <v>163</v>
+        <v>161</v>
       </c>
       <c r="D4" s="26" t="s">
         <v>61</v>
@@ -2599,16 +2600,16 @@
     </row>
     <row r="5" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A5" s="38" t="s">
-        <v>178</v>
+        <v>176</v>
       </c>
       <c r="B5" s="39" t="s">
         <v>63</v>
       </c>
       <c r="C5" s="40" t="s">
-        <v>179</v>
+        <v>177</v>
       </c>
       <c r="D5" s="39" t="s">
-        <v>180</v>
+        <v>178</v>
       </c>
       <c r="E5" s="39" t="s">
         <v>48</v>
@@ -2628,7 +2629,7 @@
         <v>63</v>
       </c>
       <c r="C6" s="40" t="s">
-        <v>164</v>
+        <v>162</v>
       </c>
       <c r="D6" s="39" t="s">
         <v>60</v>
@@ -2645,16 +2646,16 @@
     </row>
     <row r="7" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A7" s="13" t="s">
-        <v>89</v>
+        <v>87</v>
       </c>
       <c r="B7" s="26" t="s">
         <v>63</v>
       </c>
       <c r="C7" s="5" t="s">
-        <v>151</v>
+        <v>149</v>
       </c>
       <c r="D7" s="26" t="s">
-        <v>181</v>
+        <v>179</v>
       </c>
       <c r="E7" s="26" t="s">
         <v>48</v>
@@ -2668,16 +2669,16 @@
     </row>
     <row r="8" spans="1:7" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A8" s="14" t="s">
-        <v>90</v>
+        <v>88</v>
       </c>
       <c r="B8" s="27" t="s">
         <v>63</v>
       </c>
       <c r="C8" s="7" t="s">
-        <v>152</v>
+        <v>150</v>
       </c>
       <c r="D8" s="27" t="s">
-        <v>153</v>
+        <v>151</v>
       </c>
       <c r="E8" s="27" t="s">
         <v>55</v>
@@ -2700,7 +2701,7 @@
         <v>70</v>
       </c>
       <c r="D9" s="28" t="s">
-        <v>139</v>
+        <v>137</v>
       </c>
       <c r="E9" s="28" t="s">
         <v>48</v>
@@ -2726,7 +2727,7 @@
         <v>67</v>
       </c>
       <c r="E10" s="27" t="s">
-        <v>112</v>
+        <v>110</v>
       </c>
       <c r="F10" s="10">
         <v>0</v>
@@ -2740,13 +2741,13 @@
         <v>71</v>
       </c>
       <c r="B11" s="28" t="s">
-        <v>79</v>
+        <v>77</v>
       </c>
       <c r="C11" s="8" t="s">
-        <v>138</v>
+        <v>136</v>
       </c>
       <c r="D11" s="28" t="s">
-        <v>139</v>
+        <v>137</v>
       </c>
       <c r="E11" s="28" t="s">
         <v>48</v>
@@ -2763,13 +2764,13 @@
         <v>73</v>
       </c>
       <c r="B12" s="26" t="s">
-        <v>79</v>
+        <v>77</v>
       </c>
       <c r="C12" s="5" t="s">
-        <v>143</v>
+        <v>141</v>
       </c>
       <c r="D12" s="26" t="s">
-        <v>144</v>
+        <v>142</v>
       </c>
       <c r="E12" s="26" t="s">
         <v>48</v>
@@ -2786,13 +2787,13 @@
         <v>74</v>
       </c>
       <c r="B13" s="26" t="s">
-        <v>79</v>
+        <v>77</v>
       </c>
       <c r="C13" s="5" t="s">
-        <v>145</v>
+        <v>143</v>
       </c>
       <c r="D13" s="26" t="s">
-        <v>146</v>
+        <v>144</v>
       </c>
       <c r="E13" s="26" t="s">
         <v>48</v>
@@ -2809,10 +2810,10 @@
         <v>75</v>
       </c>
       <c r="B14" s="26" t="s">
-        <v>79</v>
+        <v>77</v>
       </c>
       <c r="C14" s="5" t="s">
-        <v>147</v>
+        <v>145</v>
       </c>
       <c r="D14" s="26" t="s">
         <v>61</v>
@@ -2832,13 +2833,13 @@
         <v>76</v>
       </c>
       <c r="B15" s="26" t="s">
-        <v>79</v>
+        <v>77</v>
       </c>
       <c r="C15" s="5" t="s">
-        <v>148</v>
+        <v>146</v>
       </c>
       <c r="D15" s="26" t="s">
-        <v>80</v>
+        <v>78</v>
       </c>
       <c r="E15" s="26" t="s">
         <v>48</v>
@@ -2850,58 +2851,60 @@
         <v>16</v>
       </c>
     </row>
-    <row r="16" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A16" s="13" t="s">
+    <row r="16" spans="1:7" ht="29.4" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A16" s="14" t="s">
+        <v>188</v>
+      </c>
+      <c r="B16" s="27" t="s">
         <v>77</v>
       </c>
-      <c r="B16" s="26" t="s">
+      <c r="C16" s="7" t="s">
+        <v>159</v>
+      </c>
+      <c r="D16" s="27" t="s">
+        <v>147</v>
+      </c>
+      <c r="E16" s="27" t="s">
+        <v>48</v>
+      </c>
+      <c r="F16" s="10">
+        <v>1</v>
+      </c>
+      <c r="G16" s="30" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="17" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A17" s="12" t="s">
         <v>79</v>
       </c>
-      <c r="C16" s="5"/>
-      <c r="D16" s="26" t="s">
-        <v>158</v>
-      </c>
-      <c r="E16" s="26" t="s">
+      <c r="B17" s="28" t="s">
+        <v>89</v>
+      </c>
+      <c r="C17" s="8"/>
+      <c r="D17" s="28" t="s">
+        <v>138</v>
+      </c>
+      <c r="E17" s="28" t="s">
         <v>48</v>
       </c>
-      <c r="F16" s="6">
-        <v>1</v>
-      </c>
-      <c r="G16" s="29"/>
-    </row>
-    <row r="17" spans="1:7" ht="29.4" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A17" s="14" t="s">
-        <v>78</v>
-      </c>
-      <c r="B17" s="27" t="s">
-        <v>79</v>
-      </c>
-      <c r="C17" s="7" t="s">
-        <v>161</v>
-      </c>
-      <c r="D17" s="27" t="s">
-        <v>149</v>
-      </c>
-      <c r="E17" s="27" t="s">
-        <v>48</v>
-      </c>
-      <c r="F17" s="10">
-        <v>1</v>
-      </c>
-      <c r="G17" s="30" t="s">
+      <c r="F17" s="9">
+        <v>3</v>
+      </c>
+      <c r="G17" s="31" t="s">
         <v>16</v>
       </c>
     </row>
     <row r="18" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A18" s="12" t="s">
-        <v>81</v>
-      </c>
-      <c r="B18" s="28" t="s">
-        <v>91</v>
-      </c>
-      <c r="C18" s="8"/>
-      <c r="D18" s="28" t="s">
-        <v>140</v>
+      <c r="A18" s="13" t="s">
+        <v>80</v>
+      </c>
+      <c r="B18" s="26" t="s">
+        <v>89</v>
+      </c>
+      <c r="C18" s="5"/>
+      <c r="D18" s="26" t="s">
+        <v>139</v>
       </c>
       <c r="E18" s="28" t="s">
         <v>48</v>
@@ -2909,20 +2912,20 @@
       <c r="F18" s="9">
         <v>3</v>
       </c>
-      <c r="G18" s="31" t="s">
+      <c r="G18" s="29" t="s">
         <v>16</v>
       </c>
     </row>
     <row r="19" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A19" s="13" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="B19" s="26" t="s">
-        <v>91</v>
+        <v>89</v>
       </c>
       <c r="C19" s="5"/>
       <c r="D19" s="26" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="E19" s="28" t="s">
         <v>48</v>
@@ -2934,39 +2937,39 @@
         <v>16</v>
       </c>
     </row>
-    <row r="20" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="20" spans="1:7" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A20" s="13" t="s">
-        <v>83</v>
+        <v>76</v>
       </c>
       <c r="B20" s="26" t="s">
-        <v>91</v>
-      </c>
-      <c r="C20" s="5"/>
+        <v>89</v>
+      </c>
+      <c r="C20" s="5" t="s">
+        <v>146</v>
+      </c>
       <c r="D20" s="26" t="s">
-        <v>142</v>
-      </c>
-      <c r="E20" s="28" t="s">
+        <v>78</v>
+      </c>
+      <c r="E20" s="26" t="s">
         <v>48</v>
       </c>
-      <c r="F20" s="9">
-        <v>3</v>
+      <c r="F20" s="6">
+        <v>1</v>
       </c>
       <c r="G20" s="29" t="s">
         <v>16</v>
       </c>
     </row>
-    <row r="21" spans="1:7" ht="43.2" x14ac:dyDescent="0.3">
+    <row r="21" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A21" s="13" t="s">
-        <v>76</v>
+        <v>152</v>
       </c>
       <c r="B21" s="26" t="s">
-        <v>91</v>
-      </c>
-      <c r="C21" s="5" t="s">
-        <v>148</v>
-      </c>
+        <v>89</v>
+      </c>
+      <c r="C21" s="5"/>
       <c r="D21" s="26" t="s">
-        <v>80</v>
+        <v>156</v>
       </c>
       <c r="E21" s="26" t="s">
         <v>48</v>
@@ -2974,60 +2977,60 @@
       <c r="F21" s="6">
         <v>1</v>
       </c>
-      <c r="G21" s="29" t="s">
+      <c r="G21" s="29"/>
+    </row>
+    <row r="22" spans="1:7" ht="29.4" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A22" s="14" t="s">
+        <v>153</v>
+      </c>
+      <c r="B22" s="27" t="s">
+        <v>89</v>
+      </c>
+      <c r="C22" s="7" t="s">
+        <v>159</v>
+      </c>
+      <c r="D22" s="27" t="s">
+        <v>147</v>
+      </c>
+      <c r="E22" s="27" t="s">
+        <v>48</v>
+      </c>
+      <c r="F22" s="10">
+        <v>1</v>
+      </c>
+      <c r="G22" s="30"/>
+    </row>
+    <row r="23" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A23" s="12" t="s">
+        <v>82</v>
+      </c>
+      <c r="B23" s="28" t="s">
+        <v>90</v>
+      </c>
+      <c r="C23" s="8"/>
+      <c r="D23" s="28" t="s">
+        <v>138</v>
+      </c>
+      <c r="E23" s="28" t="s">
+        <v>48</v>
+      </c>
+      <c r="F23" s="9">
+        <v>3</v>
+      </c>
+      <c r="G23" s="31" t="s">
         <v>16</v>
       </c>
     </row>
-    <row r="22" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A22" s="13" t="s">
-        <v>154</v>
-      </c>
-      <c r="B22" s="26" t="s">
-        <v>91</v>
-      </c>
-      <c r="C22" s="5"/>
-      <c r="D22" s="26" t="s">
-        <v>158</v>
-      </c>
-      <c r="E22" s="26" t="s">
-        <v>48</v>
-      </c>
-      <c r="F22" s="6">
-        <v>1</v>
-      </c>
-      <c r="G22" s="29"/>
-    </row>
-    <row r="23" spans="1:7" ht="29.4" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A23" s="14" t="s">
-        <v>155</v>
-      </c>
-      <c r="B23" s="27" t="s">
-        <v>91</v>
-      </c>
-      <c r="C23" s="7" t="s">
-        <v>161</v>
-      </c>
-      <c r="D23" s="27" t="s">
-        <v>149</v>
-      </c>
-      <c r="E23" s="27" t="s">
-        <v>48</v>
-      </c>
-      <c r="F23" s="10">
-        <v>1</v>
-      </c>
-      <c r="G23" s="30"/>
-    </row>
     <row r="24" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A24" s="12" t="s">
-        <v>84</v>
-      </c>
-      <c r="B24" s="28" t="s">
-        <v>92</v>
-      </c>
-      <c r="C24" s="8"/>
-      <c r="D24" s="28" t="s">
-        <v>140</v>
+      <c r="A24" s="13" t="s">
+        <v>83</v>
+      </c>
+      <c r="B24" s="26" t="s">
+        <v>90</v>
+      </c>
+      <c r="C24" s="5"/>
+      <c r="D24" s="26" t="s">
+        <v>139</v>
       </c>
       <c r="E24" s="28" t="s">
         <v>48</v>
@@ -3035,20 +3038,20 @@
       <c r="F24" s="9">
         <v>3</v>
       </c>
-      <c r="G24" s="31" t="s">
+      <c r="G24" s="29" t="s">
         <v>16</v>
       </c>
     </row>
     <row r="25" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A25" s="13" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="B25" s="26" t="s">
-        <v>92</v>
+        <v>90</v>
       </c>
       <c r="C25" s="5"/>
       <c r="D25" s="26" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="E25" s="28" t="s">
         <v>48</v>
@@ -3060,39 +3063,39 @@
         <v>16</v>
       </c>
     </row>
-    <row r="26" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="26" spans="1:7" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A26" s="13" t="s">
-        <v>86</v>
+        <v>76</v>
       </c>
       <c r="B26" s="26" t="s">
-        <v>92</v>
-      </c>
-      <c r="C26" s="5"/>
+        <v>90</v>
+      </c>
+      <c r="C26" s="5" t="s">
+        <v>146</v>
+      </c>
       <c r="D26" s="26" t="s">
-        <v>142</v>
-      </c>
-      <c r="E26" s="28" t="s">
+        <v>78</v>
+      </c>
+      <c r="E26" s="26" t="s">
         <v>48</v>
       </c>
-      <c r="F26" s="9">
-        <v>3</v>
+      <c r="F26" s="6">
+        <v>1</v>
       </c>
       <c r="G26" s="29" t="s">
         <v>16</v>
       </c>
     </row>
-    <row r="27" spans="1:7" ht="43.2" x14ac:dyDescent="0.3">
+    <row r="27" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A27" s="13" t="s">
-        <v>76</v>
+        <v>154</v>
       </c>
       <c r="B27" s="26" t="s">
-        <v>92</v>
-      </c>
-      <c r="C27" s="5" t="s">
-        <v>148</v>
-      </c>
+        <v>90</v>
+      </c>
+      <c r="C27" s="5"/>
       <c r="D27" s="26" t="s">
-        <v>80</v>
+        <v>156</v>
       </c>
       <c r="E27" s="26" t="s">
         <v>48</v>
@@ -3100,104 +3103,92 @@
       <c r="F27" s="6">
         <v>1</v>
       </c>
-      <c r="G27" s="29" t="s">
+      <c r="G27" s="29"/>
+    </row>
+    <row r="28" spans="1:7" ht="29.4" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A28" s="14" t="s">
+        <v>155</v>
+      </c>
+      <c r="B28" s="27" t="s">
+        <v>90</v>
+      </c>
+      <c r="C28" s="7" t="s">
+        <v>159</v>
+      </c>
+      <c r="D28" s="27" t="s">
+        <v>147</v>
+      </c>
+      <c r="E28" s="27" t="s">
+        <v>48</v>
+      </c>
+      <c r="F28" s="10">
+        <v>1</v>
+      </c>
+      <c r="G28" s="30"/>
+    </row>
+    <row r="29" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A29" s="12" t="s">
+        <v>85</v>
+      </c>
+      <c r="B29" s="28" t="s">
+        <v>91</v>
+      </c>
+      <c r="C29" s="8" t="s">
+        <v>157</v>
+      </c>
+      <c r="D29" s="28" t="s">
+        <v>137</v>
+      </c>
+      <c r="E29" s="28" t="s">
+        <v>48</v>
+      </c>
+      <c r="F29" s="9">
+        <v>3</v>
+      </c>
+      <c r="G29" s="31" t="s">
         <v>16</v>
       </c>
     </row>
-    <row r="28" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A28" s="13" t="s">
-        <v>156</v>
-      </c>
-      <c r="B28" s="26" t="s">
-        <v>92</v>
-      </c>
-      <c r="C28" s="5"/>
-      <c r="D28" s="26" t="s">
-        <v>158</v>
-      </c>
-      <c r="E28" s="26" t="s">
+    <row r="30" spans="1:7" ht="58.2" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A30" s="14" t="s">
+        <v>86</v>
+      </c>
+      <c r="B30" s="27" t="s">
+        <v>91</v>
+      </c>
+      <c r="C30" s="7" t="s">
+        <v>148</v>
+      </c>
+      <c r="D30" s="27" t="s">
+        <v>62</v>
+      </c>
+      <c r="E30" s="27" t="s">
         <v>48</v>
       </c>
-      <c r="F28" s="6">
+      <c r="F30" s="10">
         <v>1</v>
       </c>
-      <c r="G28" s="29"/>
-    </row>
-    <row r="29" spans="1:7" ht="29.4" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A29" s="14" t="s">
-        <v>157</v>
-      </c>
-      <c r="B29" s="27" t="s">
-        <v>92</v>
-      </c>
-      <c r="C29" s="7" t="s">
-        <v>161</v>
-      </c>
-      <c r="D29" s="27" t="s">
-        <v>149</v>
-      </c>
-      <c r="E29" s="27" t="s">
-        <v>48</v>
-      </c>
-      <c r="F29" s="10">
-        <v>1</v>
-      </c>
-      <c r="G29" s="30"/>
-    </row>
-    <row r="30" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A30" s="12" t="s">
-        <v>87</v>
-      </c>
-      <c r="B30" s="28" t="s">
-        <v>93</v>
-      </c>
-      <c r="C30" s="8" t="s">
-        <v>159</v>
-      </c>
-      <c r="D30" s="28" t="s">
-        <v>139</v>
-      </c>
-      <c r="E30" s="28" t="s">
-        <v>48</v>
-      </c>
-      <c r="F30" s="9">
-        <v>3</v>
-      </c>
-      <c r="G30" s="31" t="s">
+      <c r="G30" s="30" t="s">
         <v>16</v>
       </c>
     </row>
-    <row r="31" spans="1:7" ht="58.2" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A31" s="14" t="s">
-        <v>88</v>
-      </c>
-      <c r="B31" s="27" t="s">
-        <v>93</v>
-      </c>
-      <c r="C31" s="7" t="s">
-        <v>150</v>
-      </c>
-      <c r="D31" s="27" t="s">
-        <v>62</v>
-      </c>
-      <c r="E31" s="27" t="s">
-        <v>48</v>
-      </c>
-      <c r="F31" s="10">
-        <v>1</v>
-      </c>
-      <c r="G31" s="30" t="s">
-        <v>16</v>
-      </c>
+    <row r="31" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A31" s="12"/>
+      <c r="B31" s="28"/>
+      <c r="C31" s="8"/>
+      <c r="D31" s="28"/>
+      <c r="E31" s="28"/>
+      <c r="F31" s="9"/>
+      <c r="G31" s="31"/>
     </row>
     <row r="32" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A32" s="12"/>
-      <c r="B32" s="28"/>
-      <c r="C32" s="8"/>
-      <c r="D32" s="28"/>
-      <c r="E32" s="28"/>
-      <c r="F32" s="9"/>
-      <c r="G32" s="31"/>
+      <c r="A32" s="13"/>
+      <c r="B32" s="26"/>
+      <c r="C32" s="5"/>
+      <c r="D32" s="26"/>
+      <c r="E32" s="26"/>
+      <c r="F32" s="6"/>
+      <c r="G32" s="29"/>
     </row>
     <row r="33" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A33" s="13"/>
@@ -3289,27 +3280,18 @@
       <c r="F42" s="6"/>
       <c r="G42" s="29"/>
     </row>
-    <row r="43" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A43" s="13"/>
-      <c r="B43" s="26"/>
-      <c r="C43" s="5"/>
-      <c r="D43" s="26"/>
-      <c r="E43" s="26"/>
-      <c r="F43" s="6"/>
-      <c r="G43" s="29"/>
-    </row>
   </sheetData>
   <dataValidations count="8">
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="F32:F43" xr:uid="{257EC82B-68B5-4F35-825F-C289285A7C45}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="F31:F42" xr:uid="{257EC82B-68B5-4F35-825F-C289285A7C45}">
       <formula1>"fs, fel"</formula1>
     </dataValidation>
-    <dataValidation type="whole" operator="greaterThan" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="F11 F9 F18:F20 F24:F26 F30" xr:uid="{3798FD8E-D43D-4D9F-BE2C-52321394B345}">
+    <dataValidation type="whole" operator="greaterThan" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="F11 F9 F17:F19 F23:F25 F29" xr:uid="{3798FD8E-D43D-4D9F-BE2C-52321394B345}">
       <formula1>0</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="F12:F17 F21:F23 F27:F29" xr:uid="{71E12662-7031-4247-910F-BB7CE1CF6CD0}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="F20:F22 F26:F28 F12:F16" xr:uid="{71E12662-7031-4247-910F-BB7CE1CF6CD0}">
       <formula1>"1, 2"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="F31" xr:uid="{37FEDC31-329E-44E8-806D-0ED1512CF102}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="F30" xr:uid="{37FEDC31-329E-44E8-806D-0ED1512CF102}">
       <formula1>"1, 2, 3"</formula1>
     </dataValidation>
     <dataValidation type="whole" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="F7" xr:uid="{42D8AC35-50A5-40BC-BBFA-BE08B273A500}">
@@ -3509,16 +3491,16 @@
     </row>
     <row r="8" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A8" s="12" t="s">
-        <v>94</v>
+        <v>92</v>
       </c>
       <c r="B8" s="28" t="s">
         <v>23</v>
       </c>
       <c r="C8" s="8" t="s">
-        <v>175</v>
+        <v>173</v>
       </c>
       <c r="D8" s="28" t="s">
-        <v>176</v>
+        <v>174</v>
       </c>
       <c r="E8" s="28" t="s">
         <v>55</v>
@@ -3532,16 +3514,16 @@
     </row>
     <row r="9" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A9" s="13" t="s">
-        <v>95</v>
+        <v>93</v>
       </c>
       <c r="B9" s="26" t="s">
         <v>23</v>
       </c>
       <c r="C9" s="5" t="s">
-        <v>171</v>
+        <v>169</v>
       </c>
       <c r="D9" s="26" t="s">
-        <v>174</v>
+        <v>172</v>
       </c>
       <c r="E9" s="26" t="s">
         <v>49</v>
@@ -3550,21 +3532,21 @@
         <v>0</v>
       </c>
       <c r="G9" s="29" t="s">
-        <v>172</v>
+        <v>170</v>
       </c>
     </row>
     <row r="10" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A10" s="13" t="s">
-        <v>182</v>
+        <v>180</v>
       </c>
       <c r="B10" s="26" t="s">
         <v>23</v>
       </c>
       <c r="C10" s="5" t="s">
-        <v>183</v>
+        <v>181</v>
       </c>
       <c r="D10" s="26" t="s">
-        <v>184</v>
+        <v>182</v>
       </c>
       <c r="E10" s="26" t="s">
         <v>49</v>
@@ -3573,44 +3555,44 @@
         <v>0</v>
       </c>
       <c r="G10" s="29" t="s">
-        <v>172</v>
+        <v>170</v>
       </c>
     </row>
     <row r="11" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A11" s="13" t="s">
-        <v>96</v>
+        <v>94</v>
       </c>
       <c r="B11" s="26" t="s">
         <v>23</v>
       </c>
       <c r="C11" s="5" t="s">
-        <v>170</v>
+        <v>168</v>
       </c>
       <c r="D11" s="26" t="s">
-        <v>173</v>
+        <v>171</v>
       </c>
       <c r="E11" s="26" t="s">
-        <v>112</v>
+        <v>110</v>
       </c>
       <c r="F11" s="11">
         <v>20</v>
       </c>
       <c r="G11" s="29" t="s">
-        <v>169</v>
+        <v>167</v>
       </c>
     </row>
     <row r="12" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A12" s="13" t="s">
-        <v>97</v>
+        <v>95</v>
       </c>
       <c r="B12" s="26" t="s">
         <v>23</v>
       </c>
       <c r="C12" s="5" t="s">
-        <v>165</v>
+        <v>163</v>
       </c>
       <c r="D12" s="26" t="s">
-        <v>168</v>
+        <v>166</v>
       </c>
       <c r="E12" s="26" t="s">
         <v>48</v>
@@ -3624,16 +3606,16 @@
     </row>
     <row r="13" spans="1:7" ht="29.4" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A13" s="14" t="s">
-        <v>98</v>
+        <v>96</v>
       </c>
       <c r="B13" s="27" t="s">
         <v>23</v>
       </c>
       <c r="C13" s="7" t="s">
-        <v>166</v>
+        <v>164</v>
       </c>
       <c r="D13" s="27" t="s">
-        <v>167</v>
+        <v>165</v>
       </c>
       <c r="E13" s="27" t="s">
         <v>48</v>

</xml_diff>

<commit_message>
Adding Machine Learning Models
</commit_message>
<xml_diff>
--- a/config/default.xlsx
+++ b/config/default.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/f215465b21b5e6e2/Studium/34_Github/TherMOS/config/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="14" documentId="13_ncr:1_{E753D0B1-35F4-4D27-8543-876170205914}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{190F8AAD-AB2E-49F9-9BCA-764A2A64B047}"/>
+  <xr:revisionPtr revIDLastSave="113" documentId="13_ncr:1_{E753D0B1-35F4-4D27-8543-876170205914}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{03AFCBC7-35C7-4BDA-A5AC-0208E3E70427}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="30936" windowHeight="16896" activeTab="3" xr2:uid="{DB7D2548-4471-4992-93B1-3EC0BA66F7EA}"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="15360" windowHeight="16680" activeTab="3" xr2:uid="{DB7D2548-4471-4992-93B1-3EC0BA66F7EA}"/>
   </bookViews>
   <sheets>
     <sheet name="readme" sheetId="2" r:id="rId1"/>
@@ -40,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="323" uniqueCount="170">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="382" uniqueCount="201">
   <si>
     <t>#</t>
   </si>
@@ -589,6 +589,110 @@
   </si>
   <si>
     <t>Stability</t>
+  </si>
+  <si>
+    <t>Model Order KNN</t>
+  </si>
+  <si>
+    <t>knn</t>
+  </si>
+  <si>
+    <t>Number of neighbors for KNN</t>
+  </si>
+  <si>
+    <t>NSMethod</t>
+  </si>
+  <si>
+    <t>Distance Metric</t>
+  </si>
+  <si>
+    <t>Distance metric used for computing the distance of a new sample with respect to the KNN space:
+1) 'cityblock', 
+2) 'chebychev', 
+3) 'euclidean', 
+4) 'minkowski'</t>
+  </si>
+  <si>
+    <t>dist</t>
+  </si>
+  <si>
+    <t>ns</t>
+  </si>
+  <si>
+    <t>Neighbor-searcher method:
+1) 'exhaustive'
+2) 'kdtree'</t>
+  </si>
+  <si>
+    <t>MinLeafSize</t>
+  </si>
+  <si>
+    <t>MaxNumSplits</t>
+  </si>
+  <si>
+    <t>MinParentSize</t>
+  </si>
+  <si>
+    <t>leaf</t>
+  </si>
+  <si>
+    <t>split</t>
+  </si>
+  <si>
+    <t>parent</t>
+  </si>
+  <si>
+    <t>dt</t>
+  </si>
+  <si>
+    <t>Limits the maximum number of splits in the tree. This parameter directly controls the depth and complexity of the tree. Lower values reduce the tree size, potentially preventing overfitting</t>
+  </si>
+  <si>
+    <t>Specifies the minimum number of observations per leaf. Increasing MinLeafSize can reduce overfitting by preventing the tree from growing too deep</t>
+  </si>
+  <si>
+    <t>Sets the minimum number of observations in a node for it to be split. Larger values create simpler trees, as nodes with fewer observations are left unsplit.</t>
+  </si>
+  <si>
+    <t>Optimize Free Parameters</t>
+  </si>
+  <si>
+    <t>Automated optimisation of free model parameters:
+0) fixed parameters
+1) optimal parameters</t>
+  </si>
+  <si>
+    <t>opt</t>
+  </si>
+  <si>
+    <t>svm</t>
+  </si>
+  <si>
+    <t>KernelFunction</t>
+  </si>
+  <si>
+    <t>BoxConstraint</t>
+  </si>
+  <si>
+    <t>Epsilon</t>
+  </si>
+  <si>
+    <t>Sets the regularization parameter (C) that controls the trade-off between achieving a low training error and a low testing error (generalization). Higher values lead to fewer support vectors but may overfit.</t>
+  </si>
+  <si>
+    <t>Specifies the epsilon margin in the loss function, which defines a tube within which no penalty is associated with errors.</t>
+  </si>
+  <si>
+    <t>C</t>
+  </si>
+  <si>
+    <t>Specifies the kernel function to use:
+1) linear
+2) polynomial
+3) rbf</t>
+  </si>
+  <si>
+    <t>kernel</t>
   </si>
 </sst>
 </file>
@@ -662,7 +766,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="28">
+  <borders count="30">
     <border>
       <left/>
       <right/>
@@ -999,11 +1103,41 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="medium">
+        <color indexed="64"/>
+      </right>
+      <top style="medium">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="medium">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="51">
+  <cellXfs count="53">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1"/>
@@ -1124,6 +1258,12 @@
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="19" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="29" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="8" borderId="28" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -2557,156 +2697,156 @@
         <v>16</v>
       </c>
     </row>
-    <row r="7" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A7" s="13" t="s">
-        <v>81</v>
-      </c>
-      <c r="B7" s="26" t="s">
+    <row r="7" spans="1:7" ht="43.2" x14ac:dyDescent="0.3">
+      <c r="A7" s="38" t="s">
+        <v>189</v>
+      </c>
+      <c r="B7" s="39" t="s">
         <v>63</v>
       </c>
-      <c r="C7" s="5" t="s">
-        <v>136</v>
-      </c>
-      <c r="D7" s="26" t="s">
-        <v>160</v>
+      <c r="C7" s="40" t="s">
+        <v>190</v>
+      </c>
+      <c r="D7" s="39" t="s">
+        <v>191</v>
       </c>
       <c r="E7" s="26" t="s">
         <v>48</v>
       </c>
       <c r="F7" s="6">
-        <v>10</v>
+        <v>0</v>
       </c>
       <c r="G7" s="29" t="s">
         <v>16</v>
       </c>
     </row>
-    <row r="8" spans="1:7" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A8" s="14" t="s">
+    <row r="8" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A8" s="13" t="s">
+        <v>81</v>
+      </c>
+      <c r="B8" s="26" t="s">
+        <v>63</v>
+      </c>
+      <c r="C8" s="5" t="s">
+        <v>136</v>
+      </c>
+      <c r="D8" s="26" t="s">
+        <v>160</v>
+      </c>
+      <c r="E8" s="28" t="s">
+        <v>48</v>
+      </c>
+      <c r="F8" s="9">
+        <v>10</v>
+      </c>
+      <c r="G8" s="31" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="9" spans="1:7" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A9" s="14" t="s">
         <v>82</v>
       </c>
-      <c r="B8" s="27" t="s">
+      <c r="B9" s="27" t="s">
         <v>63</v>
       </c>
-      <c r="C8" s="7" t="s">
+      <c r="C9" s="7" t="s">
         <v>137</v>
       </c>
-      <c r="D8" s="27" t="s">
+      <c r="D9" s="27" t="s">
         <v>138</v>
       </c>
-      <c r="E8" s="27" t="s">
+      <c r="E9" s="27" t="s">
         <v>55</v>
       </c>
-      <c r="F8" s="42">
+      <c r="F9" s="42">
         <v>0.99990000000000001</v>
       </c>
-      <c r="G8" s="30" t="s">
+      <c r="G9" s="30" t="s">
         <v>18</v>
       </c>
     </row>
-    <row r="9" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A9" s="12" t="s">
+    <row r="10" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A10" s="12" t="s">
         <v>72</v>
       </c>
-      <c r="B9" s="28" t="s">
+      <c r="B10" s="28" t="s">
         <v>64</v>
       </c>
-      <c r="C9" s="8" t="s">
+      <c r="C10" s="8" t="s">
         <v>70</v>
       </c>
-      <c r="D9" s="28" t="s">
+      <c r="D10" s="28" t="s">
         <v>127</v>
       </c>
-      <c r="E9" s="28" t="s">
+      <c r="E10" s="28" t="s">
         <v>48</v>
       </c>
-      <c r="F9" s="9">
+      <c r="F10" s="9">
         <v>3</v>
       </c>
-      <c r="G9" s="31" t="s">
+      <c r="G10" s="31" t="s">
         <v>16</v>
       </c>
     </row>
-    <row r="10" spans="1:7" ht="29.4" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A10" s="14" t="s">
+    <row r="11" spans="1:7" ht="29.4" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A11" s="14" t="s">
         <v>66</v>
       </c>
-      <c r="B10" s="27" t="s">
+      <c r="B11" s="27" t="s">
         <v>64</v>
       </c>
-      <c r="C10" s="7" t="s">
+      <c r="C11" s="7" t="s">
         <v>68</v>
       </c>
-      <c r="D10" s="27" t="s">
+      <c r="D11" s="27" t="s">
         <v>67</v>
       </c>
-      <c r="E10" s="27" t="s">
+      <c r="E11" s="27" t="s">
         <v>102</v>
       </c>
-      <c r="F10" s="10">
+      <c r="F11" s="10">
         <v>0</v>
       </c>
-      <c r="G10" s="30" t="s">
+      <c r="G11" s="30" t="s">
         <v>69</v>
       </c>
     </row>
-    <row r="11" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A11" s="12" t="s">
+    <row r="12" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A12" s="12" t="s">
         <v>71</v>
       </c>
-      <c r="B11" s="28" t="s">
+      <c r="B12" s="28" t="s">
         <v>77</v>
       </c>
-      <c r="C11" s="8" t="s">
+      <c r="C12" s="8" t="s">
         <v>126</v>
       </c>
-      <c r="D11" s="28" t="s">
+      <c r="D12" s="28" t="s">
         <v>127</v>
       </c>
-      <c r="E11" s="28" t="s">
+      <c r="E12" s="28" t="s">
         <v>48</v>
       </c>
-      <c r="F11" s="9">
+      <c r="F12" s="9">
         <v>3</v>
       </c>
-      <c r="G11" s="31" t="s">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="12" spans="1:7" ht="43.2" x14ac:dyDescent="0.3">
-      <c r="A12" s="13" t="s">
-        <v>73</v>
-      </c>
-      <c r="B12" s="26" t="s">
-        <v>77</v>
-      </c>
-      <c r="C12" s="5" t="s">
-        <v>128</v>
-      </c>
-      <c r="D12" s="26" t="s">
-        <v>129</v>
-      </c>
-      <c r="E12" s="26" t="s">
-        <v>48</v>
-      </c>
-      <c r="F12" s="6">
-        <v>1</v>
-      </c>
-      <c r="G12" s="29" t="s">
+      <c r="G12" s="31" t="s">
         <v>16</v>
       </c>
     </row>
     <row r="13" spans="1:7" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A13" s="13" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="B13" s="26" t="s">
         <v>77</v>
       </c>
       <c r="C13" s="5" t="s">
-        <v>130</v>
+        <v>128</v>
       </c>
       <c r="D13" s="26" t="s">
-        <v>131</v>
+        <v>129</v>
       </c>
       <c r="E13" s="26" t="s">
         <v>48</v>
@@ -2718,18 +2858,18 @@
         <v>16</v>
       </c>
     </row>
-    <row r="14" spans="1:7" ht="57.6" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:7" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A14" s="13" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="B14" s="26" t="s">
         <v>77</v>
       </c>
       <c r="C14" s="5" t="s">
-        <v>132</v>
+        <v>130</v>
       </c>
       <c r="D14" s="26" t="s">
-        <v>61</v>
+        <v>131</v>
       </c>
       <c r="E14" s="26" t="s">
         <v>48</v>
@@ -2741,187 +2881,325 @@
         <v>16</v>
       </c>
     </row>
-    <row r="15" spans="1:7" ht="43.2" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:7" ht="57.6" x14ac:dyDescent="0.3">
       <c r="A15" s="13" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="B15" s="26" t="s">
         <v>77</v>
       </c>
       <c r="C15" s="5" t="s">
-        <v>133</v>
+        <v>132</v>
       </c>
       <c r="D15" s="26" t="s">
-        <v>78</v>
+        <v>61</v>
       </c>
       <c r="E15" s="26" t="s">
         <v>48</v>
       </c>
       <c r="F15" s="6">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="G15" s="29" t="s">
         <v>16</v>
       </c>
     </row>
-    <row r="16" spans="1:7" ht="29.4" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A16" s="14" t="s">
+    <row r="16" spans="1:7" ht="43.2" x14ac:dyDescent="0.3">
+      <c r="A16" s="13" t="s">
+        <v>76</v>
+      </c>
+      <c r="B16" s="26" t="s">
+        <v>77</v>
+      </c>
+      <c r="C16" s="5" t="s">
+        <v>133</v>
+      </c>
+      <c r="D16" s="26" t="s">
+        <v>78</v>
+      </c>
+      <c r="E16" s="26" t="s">
+        <v>48</v>
+      </c>
+      <c r="F16" s="6">
+        <v>2</v>
+      </c>
+      <c r="G16" s="29" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="17" spans="1:7" ht="29.4" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A17" s="14" t="s">
         <v>169</v>
       </c>
-      <c r="B16" s="27" t="s">
+      <c r="B17" s="27" t="s">
         <v>77</v>
       </c>
-      <c r="C16" s="7" t="s">
+      <c r="C17" s="7" t="s">
         <v>141</v>
       </c>
-      <c r="D16" s="27" t="s">
+      <c r="D17" s="27" t="s">
         <v>134</v>
       </c>
-      <c r="E16" s="27" t="s">
+      <c r="E17" s="27" t="s">
         <v>48</v>
       </c>
-      <c r="F16" s="10">
+      <c r="F17" s="10">
         <v>1</v>
       </c>
-      <c r="G16" s="30" t="s">
+      <c r="G17" s="30" t="s">
         <v>16</v>
       </c>
     </row>
-    <row r="17" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A17" s="12" t="s">
+    <row r="18" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A18" s="12" t="s">
         <v>79</v>
       </c>
-      <c r="B17" s="28" t="s">
+      <c r="B18" s="28" t="s">
         <v>83</v>
       </c>
-      <c r="C17" s="8" t="s">
+      <c r="C18" s="8" t="s">
         <v>139</v>
       </c>
-      <c r="D17" s="28" t="s">
+      <c r="D18" s="28" t="s">
         <v>127</v>
       </c>
-      <c r="E17" s="28" t="s">
+      <c r="E18" s="28" t="s">
         <v>48</v>
       </c>
-      <c r="F17" s="9">
+      <c r="F18" s="9">
         <v>3</v>
       </c>
-      <c r="G17" s="31" t="s">
+      <c r="G18" s="31" t="s">
         <v>16</v>
       </c>
     </row>
-    <row r="18" spans="1:7" ht="58.2" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A18" s="14" t="s">
+    <row r="19" spans="1:7" ht="58.2" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A19" s="14" t="s">
         <v>80</v>
       </c>
-      <c r="B18" s="27" t="s">
+      <c r="B19" s="27" t="s">
         <v>83</v>
       </c>
-      <c r="C18" s="7" t="s">
+      <c r="C19" s="7" t="s">
         <v>135</v>
       </c>
-      <c r="D18" s="27" t="s">
+      <c r="D19" s="27" t="s">
         <v>62</v>
       </c>
-      <c r="E18" s="27" t="s">
+      <c r="E19" s="27" t="s">
         <v>48</v>
       </c>
-      <c r="F18" s="10">
+      <c r="F19" s="10">
         <v>1</v>
       </c>
-      <c r="G18" s="30" t="s">
+      <c r="G19" s="30" t="s">
         <v>16</v>
       </c>
     </row>
-    <row r="19" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A19" s="12"/>
-      <c r="B19" s="28"/>
-      <c r="C19" s="8"/>
-      <c r="D19" s="28"/>
-      <c r="E19" s="28"/>
-      <c r="F19" s="9"/>
-      <c r="G19" s="31"/>
-    </row>
     <row r="20" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A20" s="13"/>
-      <c r="B20" s="26"/>
-      <c r="C20" s="5"/>
-      <c r="D20" s="26"/>
-      <c r="E20" s="26"/>
-      <c r="F20" s="6"/>
-      <c r="G20" s="29"/>
-    </row>
-    <row r="21" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A21" s="13"/>
-      <c r="B21" s="26"/>
-      <c r="C21" s="5"/>
-      <c r="D21" s="26"/>
-      <c r="E21" s="26"/>
-      <c r="F21" s="6"/>
+      <c r="A20" s="12" t="s">
+        <v>170</v>
+      </c>
+      <c r="B20" s="28" t="s">
+        <v>171</v>
+      </c>
+      <c r="C20" s="8" t="s">
+        <v>172</v>
+      </c>
+      <c r="D20" s="28" t="s">
+        <v>127</v>
+      </c>
+      <c r="E20" s="28" t="s">
+        <v>48</v>
+      </c>
+      <c r="F20" s="9">
+        <v>3</v>
+      </c>
+      <c r="G20" s="31" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="21" spans="1:7" ht="43.2" x14ac:dyDescent="0.3">
+      <c r="A21" s="13" t="s">
+        <v>173</v>
+      </c>
+      <c r="B21" s="26" t="s">
+        <v>171</v>
+      </c>
+      <c r="C21" s="5" t="s">
+        <v>178</v>
+      </c>
+      <c r="D21" s="26" t="s">
+        <v>177</v>
+      </c>
+      <c r="E21" s="26" t="s">
+        <v>48</v>
+      </c>
+      <c r="F21" s="6">
+        <v>1</v>
+      </c>
       <c r="G21" s="29"/>
     </row>
-    <row r="22" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A22" s="13"/>
-      <c r="B22" s="26"/>
-      <c r="C22" s="5"/>
-      <c r="D22" s="26"/>
-      <c r="E22" s="26"/>
-      <c r="F22" s="6"/>
-      <c r="G22" s="29"/>
-    </row>
-    <row r="23" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A23" s="13"/>
-      <c r="B23" s="26"/>
-      <c r="C23" s="5"/>
-      <c r="D23" s="26"/>
-      <c r="E23" s="26"/>
-      <c r="F23" s="6"/>
-      <c r="G23" s="29"/>
-    </row>
-    <row r="24" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A24" s="13"/>
-      <c r="B24" s="26"/>
-      <c r="C24" s="5"/>
-      <c r="D24" s="26"/>
-      <c r="E24" s="26"/>
-      <c r="F24" s="6"/>
-      <c r="G24" s="29"/>
-    </row>
-    <row r="25" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A25" s="13"/>
-      <c r="B25" s="26"/>
-      <c r="C25" s="5"/>
-      <c r="D25" s="26"/>
-      <c r="E25" s="26"/>
-      <c r="F25" s="6"/>
-      <c r="G25" s="29"/>
-    </row>
-    <row r="26" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A26" s="13"/>
-      <c r="B26" s="26"/>
-      <c r="C26" s="5"/>
-      <c r="D26" s="26"/>
-      <c r="E26" s="26"/>
-      <c r="F26" s="6"/>
-      <c r="G26" s="29"/>
-    </row>
-    <row r="27" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A27" s="13"/>
-      <c r="B27" s="26"/>
-      <c r="C27" s="5"/>
-      <c r="D27" s="26"/>
-      <c r="E27" s="26"/>
-      <c r="F27" s="6"/>
-      <c r="G27" s="29"/>
-    </row>
-    <row r="28" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A28" s="13"/>
-      <c r="B28" s="26"/>
-      <c r="C28" s="5"/>
-      <c r="D28" s="26"/>
-      <c r="E28" s="26"/>
-      <c r="F28" s="6"/>
-      <c r="G28" s="29"/>
+    <row r="22" spans="1:7" ht="86.4" x14ac:dyDescent="0.3">
+      <c r="A22" s="13" t="s">
+        <v>174</v>
+      </c>
+      <c r="B22" s="26" t="s">
+        <v>171</v>
+      </c>
+      <c r="C22" s="5" t="s">
+        <v>175</v>
+      </c>
+      <c r="D22" s="26" t="s">
+        <v>176</v>
+      </c>
+      <c r="E22" s="26" t="s">
+        <v>47</v>
+      </c>
+      <c r="F22" s="6">
+        <v>3</v>
+      </c>
+      <c r="G22" s="29" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="23" spans="1:7" ht="43.2" x14ac:dyDescent="0.3">
+      <c r="A23" s="12" t="s">
+        <v>179</v>
+      </c>
+      <c r="B23" s="28" t="s">
+        <v>185</v>
+      </c>
+      <c r="C23" s="8" t="s">
+        <v>187</v>
+      </c>
+      <c r="D23" s="28" t="s">
+        <v>182</v>
+      </c>
+      <c r="E23" s="28" t="s">
+        <v>48</v>
+      </c>
+      <c r="F23" s="9">
+        <v>10</v>
+      </c>
+      <c r="G23" s="31" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="24" spans="1:7" ht="57.6" x14ac:dyDescent="0.3">
+      <c r="A24" s="13" t="s">
+        <v>180</v>
+      </c>
+      <c r="B24" s="26" t="s">
+        <v>185</v>
+      </c>
+      <c r="C24" s="5" t="s">
+        <v>186</v>
+      </c>
+      <c r="D24" s="26" t="s">
+        <v>183</v>
+      </c>
+      <c r="E24" s="26" t="s">
+        <v>48</v>
+      </c>
+      <c r="F24" s="6">
+        <v>50</v>
+      </c>
+      <c r="G24" s="29" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="25" spans="1:7" ht="43.8" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A25" s="14" t="s">
+        <v>181</v>
+      </c>
+      <c r="B25" s="27" t="s">
+        <v>185</v>
+      </c>
+      <c r="C25" s="7" t="s">
+        <v>188</v>
+      </c>
+      <c r="D25" s="27" t="s">
+        <v>184</v>
+      </c>
+      <c r="E25" s="27" t="s">
+        <v>48</v>
+      </c>
+      <c r="F25" s="10">
+        <v>20</v>
+      </c>
+      <c r="G25" s="30" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="26" spans="1:7" ht="57.6" x14ac:dyDescent="0.3">
+      <c r="A26" s="12" t="s">
+        <v>193</v>
+      </c>
+      <c r="B26" s="28" t="s">
+        <v>192</v>
+      </c>
+      <c r="C26" s="8" t="s">
+        <v>199</v>
+      </c>
+      <c r="D26" s="28" t="s">
+        <v>200</v>
+      </c>
+      <c r="E26" s="28" t="s">
+        <v>47</v>
+      </c>
+      <c r="F26" s="51">
+        <v>1</v>
+      </c>
+      <c r="G26" s="52" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="27" spans="1:7" ht="57.6" x14ac:dyDescent="0.3">
+      <c r="A27" s="13" t="s">
+        <v>194</v>
+      </c>
+      <c r="B27" s="26" t="s">
+        <v>192</v>
+      </c>
+      <c r="C27" s="5" t="s">
+        <v>196</v>
+      </c>
+      <c r="D27" s="26" t="s">
+        <v>198</v>
+      </c>
+      <c r="E27" s="26" t="s">
+        <v>49</v>
+      </c>
+      <c r="F27" s="9">
+        <v>1</v>
+      </c>
+      <c r="G27" s="31" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="28" spans="1:7" ht="43.2" x14ac:dyDescent="0.3">
+      <c r="A28" s="13" t="s">
+        <v>195</v>
+      </c>
+      <c r="B28" s="26" t="s">
+        <v>192</v>
+      </c>
+      <c r="C28" s="5" t="s">
+        <v>197</v>
+      </c>
+      <c r="D28" s="26" t="s">
+        <v>20</v>
+      </c>
+      <c r="E28" s="26" t="s">
+        <v>49</v>
+      </c>
+      <c r="F28" s="6">
+        <v>1</v>
+      </c>
+      <c r="G28" s="29" t="s">
+        <v>16</v>
+      </c>
     </row>
     <row r="29" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A29" s="13"/>
@@ -2942,24 +3220,24 @@
       <c r="G30" s="29"/>
     </row>
   </sheetData>
-  <dataValidations count="8">
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="F19:F30" xr:uid="{257EC82B-68B5-4F35-825F-C289285A7C45}">
+  <dataValidations count="12">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="F29:F30" xr:uid="{257EC82B-68B5-4F35-825F-C289285A7C45}">
       <formula1>"fs, fel"</formula1>
     </dataValidation>
-    <dataValidation type="whole" operator="greaterThan" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="F11 F9 F17" xr:uid="{3798FD8E-D43D-4D9F-BE2C-52321394B345}">
+    <dataValidation type="whole" operator="greaterThan" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="F12 F10 F18 F20 F25 F23" xr:uid="{3798FD8E-D43D-4D9F-BE2C-52321394B345}">
       <formula1>0</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="F12:F16" xr:uid="{71E12662-7031-4247-910F-BB7CE1CF6CD0}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="F13:F17 F21" xr:uid="{71E12662-7031-4247-910F-BB7CE1CF6CD0}">
       <formula1>"1, 2"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="F18" xr:uid="{37FEDC31-329E-44E8-806D-0ED1512CF102}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="F19 F26" xr:uid="{37FEDC31-329E-44E8-806D-0ED1512CF102}">
       <formula1>"1, 2, 3"</formula1>
     </dataValidation>
-    <dataValidation type="whole" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="F7" xr:uid="{42D8AC35-50A5-40BC-BBFA-BE08B273A500}">
+    <dataValidation type="whole" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="F8" xr:uid="{42D8AC35-50A5-40BC-BBFA-BE08B273A500}">
       <formula1>1</formula1>
       <formula2>20</formula2>
     </dataValidation>
-    <dataValidation type="decimal" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="F2:F3 F8" xr:uid="{2B8FFCC1-6704-4765-8AD4-006A185633FA}">
+    <dataValidation type="decimal" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="F2:F3 F9" xr:uid="{2B8FFCC1-6704-4765-8AD4-006A185633FA}">
       <formula1>0</formula1>
       <formula2>1</formula2>
     </dataValidation>
@@ -2969,6 +3247,18 @@
     <dataValidation type="whole" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="F5:F6" xr:uid="{F4E45863-F6B6-49B0-9AF0-77CB1F5B4777}">
       <formula1>10</formula1>
       <formula2>1000000</formula2>
+    </dataValidation>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="F7" xr:uid="{6B215F84-9F1B-41AC-8192-16AB63AE3266}">
+      <formula1>"0, 1"</formula1>
+    </dataValidation>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="F22" xr:uid="{47B450A3-D6D0-4908-B7DA-713464E39E93}">
+      <formula1>"1, 2, 3, 4"</formula1>
+    </dataValidation>
+    <dataValidation type="whole" operator="greaterThan" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="F24" xr:uid="{4036D9AA-DD26-43F2-86CA-83C98477498F}">
+      <formula1>1</formula1>
+    </dataValidation>
+    <dataValidation type="decimal" operator="greaterThan" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="F27:F28" xr:uid="{E87A8820-6156-4E10-8AF9-95041973A5CF}">
+      <formula1>0</formula1>
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
Adding Machine and Deep Learning Structures
</commit_message>
<xml_diff>
--- a/config/default.xlsx
+++ b/config/default.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/f215465b21b5e6e2/Studium/34_Github/TherMOS/config/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="113" documentId="13_ncr:1_{E753D0B1-35F4-4D27-8543-876170205914}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{03AFCBC7-35C7-4BDA-A5AC-0208E3E70427}"/>
+  <xr:revisionPtr revIDLastSave="189" documentId="13_ncr:1_{E753D0B1-35F4-4D27-8543-876170205914}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{78A8A145-736B-4EB8-8914-66ECAF6B1CC9}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="15360" windowHeight="16680" activeTab="3" xr2:uid="{DB7D2548-4471-4992-93B1-3EC0BA66F7EA}"/>
+    <workbookView xWindow="732" yWindow="4476" windowWidth="23040" windowHeight="12204" activeTab="1" xr2:uid="{DB7D2548-4471-4992-93B1-3EC0BA66F7EA}"/>
   </bookViews>
   <sheets>
     <sheet name="readme" sheetId="2" r:id="rId1"/>
@@ -40,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="382" uniqueCount="201">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="436" uniqueCount="229">
   <si>
     <t>#</t>
   </si>
@@ -693,6 +693,93 @@
   </si>
   <si>
     <t>kernel</t>
+  </si>
+  <si>
+    <t>MaxEpochs</t>
+  </si>
+  <si>
+    <t>GradientThreshold</t>
+  </si>
+  <si>
+    <t>InitialLearnRate</t>
+  </si>
+  <si>
+    <t>LearnRateDropPeriod</t>
+  </si>
+  <si>
+    <t>LearnRateDropFactor</t>
+  </si>
+  <si>
+    <t>ValidationFrequency</t>
+  </si>
+  <si>
+    <t>dl</t>
+  </si>
+  <si>
+    <t>MiniBatchSize</t>
+  </si>
+  <si>
+    <t>Shuffle</t>
+  </si>
+  <si>
+    <t>ValidationPatience</t>
+  </si>
+  <si>
+    <t>Specifies the maximum number of passes through the entire training dataset. Higher values can lead to better training but also increase the risk of overfitting.</t>
+  </si>
+  <si>
+    <t>Specifies the threshold for gradient clipping to prevent the gradients from exploding. It's useful when training deep networks.</t>
+  </si>
+  <si>
+    <t>epoch</t>
+  </si>
+  <si>
+    <t>gradTh</t>
+  </si>
+  <si>
+    <t>initLr</t>
+  </si>
+  <si>
+    <t>The initial step size for updating the weights. A higher value may speed up learning but can cause instability, while a lower value ensures stable convergence.</t>
+  </si>
+  <si>
+    <t>Specifies the number of epochs between reductions of the learning rate when using the 'piecewise' schedule.</t>
+  </si>
+  <si>
+    <t>Specifies the factor by which the learning rate is reduced. For example, a value of 0.2 means the learning rate is multiplied by 0.2 (i.e., reduced by 80%).</t>
+  </si>
+  <si>
+    <t>lrDropPr</t>
+  </si>
+  <si>
+    <t>lrDropFa</t>
+  </si>
+  <si>
+    <t>Specifies the frequency (in iterations) at which the validation performance is computed. This helps in early stopping and monitoring the progress.</t>
+  </si>
+  <si>
+    <t>valFreq</t>
+  </si>
+  <si>
+    <t>Specifies the number of observations to use in each mini-batch. Smaller sizes can reduce memory usage and allow for more frequent updates.</t>
+  </si>
+  <si>
+    <t>batch</t>
+  </si>
+  <si>
+    <t>Specifies how to shuffle the data before each epoch. Options include 'never', 'once', and 'every-epoch':
+1) never
+2) once
+3) every-epoch</t>
+  </si>
+  <si>
+    <t>shu</t>
+  </si>
+  <si>
+    <t>Specifies the number of epochs with no improvement on the validation data before training is stopped.</t>
+  </si>
+  <si>
+    <t>valPat</t>
   </si>
 </sst>
 </file>
@@ -1250,6 +1337,12 @@
     <xf numFmtId="0" fontId="0" fillId="4" borderId="26" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="29" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="8" borderId="28" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -1258,12 +1351,6 @@
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="19" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="29" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="8" borderId="28" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -1646,11 +1733,11 @@
       <c r="F13" s="1" t="s">
         <v>12</v>
       </c>
-      <c r="J13" s="48" t="s">
+      <c r="J13" s="50" t="s">
         <v>24</v>
       </c>
-      <c r="K13" s="49"/>
-      <c r="L13" s="50"/>
+      <c r="K13" s="51"/>
+      <c r="L13" s="52"/>
     </row>
     <row r="14" spans="1:12" ht="15.6" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A14" s="3">
@@ -2549,7 +2636,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{799FBFCB-8244-4B83-8CC9-EBD2890613E5}">
-  <dimension ref="A1:G30"/>
+  <dimension ref="A1:G41"/>
   <sheetFormatPr defaultColWidth="9.109375" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="29.33203125" bestFit="1" customWidth="1"/>
@@ -3148,10 +3235,10 @@
       <c r="E26" s="28" t="s">
         <v>47</v>
       </c>
-      <c r="F26" s="51">
+      <c r="F26" s="48">
         <v>1</v>
       </c>
-      <c r="G26" s="52" t="s">
+      <c r="G26" s="49" t="s">
         <v>16</v>
       </c>
     </row>
@@ -3178,50 +3265,275 @@
         <v>16</v>
       </c>
     </row>
-    <row r="28" spans="1:7" ht="43.2" x14ac:dyDescent="0.3">
-      <c r="A28" s="13" t="s">
+    <row r="28" spans="1:7" ht="43.8" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A28" s="14" t="s">
         <v>195</v>
       </c>
-      <c r="B28" s="26" t="s">
+      <c r="B28" s="27" t="s">
         <v>192</v>
       </c>
-      <c r="C28" s="5" t="s">
+      <c r="C28" s="7" t="s">
         <v>197</v>
       </c>
-      <c r="D28" s="26" t="s">
+      <c r="D28" s="27" t="s">
         <v>20</v>
       </c>
-      <c r="E28" s="26" t="s">
+      <c r="E28" s="27" t="s">
         <v>49</v>
       </c>
-      <c r="F28" s="6">
+      <c r="F28" s="10">
         <v>1</v>
       </c>
-      <c r="G28" s="29" t="s">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="29" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A29" s="13"/>
-      <c r="B29" s="26"/>
-      <c r="C29" s="5"/>
-      <c r="D29" s="26"/>
-      <c r="E29" s="26"/>
-      <c r="F29" s="6"/>
-      <c r="G29" s="29"/>
-    </row>
-    <row r="30" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A30" s="13"/>
-      <c r="B30" s="26"/>
-      <c r="C30" s="5"/>
-      <c r="D30" s="26"/>
-      <c r="E30" s="26"/>
-      <c r="F30" s="6"/>
-      <c r="G30" s="29"/>
+      <c r="G28" s="30" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="29" spans="1:7" ht="43.2" x14ac:dyDescent="0.3">
+      <c r="A29" s="12" t="s">
+        <v>201</v>
+      </c>
+      <c r="B29" s="28" t="s">
+        <v>207</v>
+      </c>
+      <c r="C29" s="8" t="s">
+        <v>211</v>
+      </c>
+      <c r="D29" s="28" t="s">
+        <v>213</v>
+      </c>
+      <c r="E29" s="26" t="s">
+        <v>48</v>
+      </c>
+      <c r="F29" s="6">
+        <v>100</v>
+      </c>
+      <c r="G29" s="29" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="30" spans="1:7" ht="43.2" x14ac:dyDescent="0.3">
+      <c r="A30" s="13" t="s">
+        <v>202</v>
+      </c>
+      <c r="B30" s="26" t="s">
+        <v>207</v>
+      </c>
+      <c r="C30" s="5" t="s">
+        <v>212</v>
+      </c>
+      <c r="D30" s="26" t="s">
+        <v>214</v>
+      </c>
+      <c r="E30" s="26" t="s">
+        <v>49</v>
+      </c>
+      <c r="F30" s="9">
+        <v>1</v>
+      </c>
+      <c r="G30" s="31" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="31" spans="1:7" ht="43.2" x14ac:dyDescent="0.3">
+      <c r="A31" s="13" t="s">
+        <v>203</v>
+      </c>
+      <c r="B31" s="26" t="s">
+        <v>207</v>
+      </c>
+      <c r="C31" s="5" t="s">
+        <v>216</v>
+      </c>
+      <c r="D31" s="26" t="s">
+        <v>215</v>
+      </c>
+      <c r="E31" s="26" t="s">
+        <v>49</v>
+      </c>
+      <c r="F31" s="9">
+        <v>5.0000000000000001E-3</v>
+      </c>
+      <c r="G31" s="31" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="32" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A32" s="13" t="s">
+        <v>204</v>
+      </c>
+      <c r="B32" s="26" t="s">
+        <v>207</v>
+      </c>
+      <c r="C32" s="5" t="s">
+        <v>217</v>
+      </c>
+      <c r="D32" s="26" t="s">
+        <v>219</v>
+      </c>
+      <c r="E32" s="26" t="s">
+        <v>48</v>
+      </c>
+      <c r="F32" s="6">
+        <v>50</v>
+      </c>
+      <c r="G32" s="31" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="33" spans="1:7" ht="43.2" x14ac:dyDescent="0.3">
+      <c r="A33" s="13" t="s">
+        <v>205</v>
+      </c>
+      <c r="B33" s="26" t="s">
+        <v>207</v>
+      </c>
+      <c r="C33" s="5" t="s">
+        <v>218</v>
+      </c>
+      <c r="D33" s="26" t="s">
+        <v>220</v>
+      </c>
+      <c r="E33" s="26" t="s">
+        <v>49</v>
+      </c>
+      <c r="F33" s="9">
+        <v>0.2</v>
+      </c>
+      <c r="G33" s="29" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="34" spans="1:7" ht="43.2" x14ac:dyDescent="0.3">
+      <c r="A34" s="13" t="s">
+        <v>206</v>
+      </c>
+      <c r="B34" s="26" t="s">
+        <v>207</v>
+      </c>
+      <c r="C34" s="5" t="s">
+        <v>221</v>
+      </c>
+      <c r="D34" s="26" t="s">
+        <v>222</v>
+      </c>
+      <c r="E34" s="26" t="s">
+        <v>48</v>
+      </c>
+      <c r="F34" s="6">
+        <v>10</v>
+      </c>
+      <c r="G34" s="29" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="35" spans="1:7" ht="43.2" x14ac:dyDescent="0.3">
+      <c r="A35" s="13" t="s">
+        <v>208</v>
+      </c>
+      <c r="B35" s="26" t="s">
+        <v>207</v>
+      </c>
+      <c r="C35" s="5" t="s">
+        <v>223</v>
+      </c>
+      <c r="D35" s="26" t="s">
+        <v>224</v>
+      </c>
+      <c r="E35" s="26" t="s">
+        <v>48</v>
+      </c>
+      <c r="F35" s="6">
+        <v>64</v>
+      </c>
+      <c r="G35" s="29" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="36" spans="1:7" ht="72" x14ac:dyDescent="0.3">
+      <c r="A36" s="13" t="s">
+        <v>209</v>
+      </c>
+      <c r="B36" s="26" t="s">
+        <v>207</v>
+      </c>
+      <c r="C36" s="5" t="s">
+        <v>225</v>
+      </c>
+      <c r="D36" s="26" t="s">
+        <v>226</v>
+      </c>
+      <c r="E36" s="26" t="s">
+        <v>48</v>
+      </c>
+      <c r="F36" s="6">
+        <v>1</v>
+      </c>
+      <c r="G36" s="29" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="37" spans="1:7" ht="29.4" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A37" s="14" t="s">
+        <v>210</v>
+      </c>
+      <c r="B37" s="27" t="s">
+        <v>207</v>
+      </c>
+      <c r="C37" s="7" t="s">
+        <v>227</v>
+      </c>
+      <c r="D37" s="27" t="s">
+        <v>228</v>
+      </c>
+      <c r="E37" s="27" t="s">
+        <v>48</v>
+      </c>
+      <c r="F37" s="10">
+        <v>5</v>
+      </c>
+      <c r="G37" s="30" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="38" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A38" s="12"/>
+      <c r="B38" s="28"/>
+      <c r="C38" s="8"/>
+      <c r="D38" s="28"/>
+      <c r="E38" s="28"/>
+      <c r="F38" s="9"/>
+      <c r="G38" s="31"/>
+    </row>
+    <row r="39" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A39" s="13"/>
+      <c r="B39" s="26"/>
+      <c r="C39" s="5"/>
+      <c r="D39" s="26"/>
+      <c r="E39" s="26"/>
+      <c r="F39" s="6"/>
+      <c r="G39" s="29"/>
+    </row>
+    <row r="40" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A40" s="13"/>
+      <c r="B40" s="26"/>
+      <c r="C40" s="5"/>
+      <c r="D40" s="26"/>
+      <c r="E40" s="26"/>
+      <c r="F40" s="6"/>
+      <c r="G40" s="29"/>
+    </row>
+    <row r="41" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A41" s="13"/>
+      <c r="B41" s="26"/>
+      <c r="C41" s="5"/>
+      <c r="D41" s="26"/>
+      <c r="E41" s="26"/>
+      <c r="F41" s="6"/>
+      <c r="G41" s="29"/>
     </row>
   </sheetData>
   <dataValidations count="12">
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="F29:F30" xr:uid="{257EC82B-68B5-4F35-825F-C289285A7C45}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="F38:F41" xr:uid="{257EC82B-68B5-4F35-825F-C289285A7C45}">
       <formula1>"fs, fel"</formula1>
     </dataValidation>
     <dataValidation type="whole" operator="greaterThan" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="F12 F10 F18 F20 F25 F23" xr:uid="{3798FD8E-D43D-4D9F-BE2C-52321394B345}">
@@ -3230,7 +3542,7 @@
     <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="F13:F17 F21" xr:uid="{71E12662-7031-4247-910F-BB7CE1CF6CD0}">
       <formula1>"1, 2"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="F19 F26" xr:uid="{37FEDC31-329E-44E8-806D-0ED1512CF102}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="F19 F26 F36" xr:uid="{37FEDC31-329E-44E8-806D-0ED1512CF102}">
       <formula1>"1, 2, 3"</formula1>
     </dataValidation>
     <dataValidation type="whole" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="F8" xr:uid="{42D8AC35-50A5-40BC-BBFA-BE08B273A500}">
@@ -3254,10 +3566,10 @@
     <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="F22" xr:uid="{47B450A3-D6D0-4908-B7DA-713464E39E93}">
       <formula1>"1, 2, 3, 4"</formula1>
     </dataValidation>
-    <dataValidation type="whole" operator="greaterThan" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="F24" xr:uid="{4036D9AA-DD26-43F2-86CA-83C98477498F}">
+    <dataValidation type="whole" operator="greaterThan" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="F24 F29 F37 F32 F34:F35" xr:uid="{4036D9AA-DD26-43F2-86CA-83C98477498F}">
       <formula1>1</formula1>
     </dataValidation>
-    <dataValidation type="decimal" operator="greaterThan" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="F27:F28" xr:uid="{E87A8820-6156-4E10-8AF9-95041973A5CF}">
+    <dataValidation type="decimal" operator="greaterThan" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="F27:F28 F30:F31 F33" xr:uid="{E87A8820-6156-4E10-8AF9-95041973A5CF}">
       <formula1>0</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>